<commit_message>
Update industry raw data workbook
</commit_message>
<xml_diff>
--- a/data/raw/data_industry.xlsx
+++ b/data/raw/data_industry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kande\Documents\GitHub\Industry_optimisation_model\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560780B8-8624-4AA0-9903-6D9D91AD7B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FA4688D-E305-4E77-84E4-96223AC9B23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="17520" xr2:uid="{69F55029-E6FD-4DAD-9766-3BCD230AD838}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="10" xr2:uid="{69F55029-E6FD-4DAD-9766-3BCD230AD838}"/>
   </bookViews>
   <sheets>
     <sheet name="prices" sheetId="5" r:id="rId1"/>
@@ -37,6 +37,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">prices!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -9008,11 +9009,11 @@
         <v>152</v>
       </c>
       <c r="C4" s="71">
-        <f t="shared" ref="C4:D4" si="0">160*C2+0</f>
+        <f>160*C2+0</f>
         <v>80</v>
       </c>
       <c r="D4" s="71">
-        <f t="shared" si="0"/>
+        <f>160*D2+0</f>
         <v>119.19999999999999</v>
       </c>
       <c r="E4" s="73">
@@ -9267,19 +9268,19 @@
         <v>0.95</v>
       </c>
       <c r="C8">
-        <f t="shared" ref="C8:F8" si="0">C2+C3</f>
+        <f>C2+C3</f>
         <v>0.7</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
+        <f>D2+D3</f>
         <v>0.74499999999999988</v>
       </c>
       <c r="E8">
-        <f t="shared" si="0"/>
+        <f>E2+E3</f>
         <v>0.5</v>
       </c>
       <c r="F8">
-        <f t="shared" si="0"/>
+        <f>F2+F3</f>
         <v>0.65</v>
       </c>
     </row>

</xml_diff>